<commit_message>
Update! PCB and old stuff!
</commit_message>
<xml_diff>
--- a/PCB/BOM_Board1_PCB1_2026-08-11.xlsx
+++ b/PCB/BOM_Board1_PCB1_2026-08-11.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="207">
   <si>
     <t>No.</t>
   </si>
@@ -400,6 +400,21 @@
     <t>20</t>
   </si>
   <si>
+    <t>5.1kΩ</t>
+  </si>
+  <si>
+    <t>R12</t>
+  </si>
+  <si>
+    <t>FRC0402J512 TS</t>
+  </si>
+  <si>
+    <t>C2906948</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
     <t>TS-1187A-B-A-B</t>
   </si>
   <si>
@@ -415,7 +430,7 @@
     <t>C318884</t>
   </si>
   <si>
-    <t>21</t>
+    <t>22</t>
   </si>
   <si>
     <t>RP2350B</t>
@@ -433,7 +448,7 @@
     <t>C42415655</t>
   </si>
   <si>
-    <t>22</t>
+    <t>23</t>
   </si>
   <si>
     <t>BNO055</t>
@@ -451,7 +466,7 @@
     <t>C93216</t>
   </si>
   <si>
-    <t>23</t>
+    <t>24</t>
   </si>
   <si>
     <t>BME680</t>
@@ -466,7 +481,7 @@
     <t>C125972</t>
   </si>
   <si>
-    <t>24</t>
+    <t>25</t>
   </si>
   <si>
     <t>INA226AIDGSR</t>
@@ -484,7 +499,7 @@
     <t>C49851</t>
   </si>
   <si>
-    <t>25</t>
+    <t>26</t>
   </si>
   <si>
     <t>LIS3MDLTR</t>
@@ -502,7 +517,7 @@
     <t>C478483</t>
   </si>
   <si>
-    <t>26</t>
+    <t>27</t>
   </si>
   <si>
     <t>AP2112K-3.3TRG1</t>
@@ -520,7 +535,7 @@
     <t>C23380830</t>
   </si>
   <si>
-    <t>27</t>
+    <t>28</t>
   </si>
   <si>
     <t>B3B-XH-A(LF)(SN)</t>
@@ -535,7 +550,7 @@
     <t>C144394</t>
   </si>
   <si>
-    <t>28</t>
+    <t>29</t>
   </si>
   <si>
     <t>12MHz</t>
@@ -553,7 +568,7 @@
     <t>C20625731</t>
   </si>
   <si>
-    <t>29</t>
+    <t>30</t>
   </si>
   <si>
     <t>SS-12D00-G3</t>
@@ -571,7 +586,7 @@
     <t>C22355741</t>
   </si>
   <si>
-    <t>30</t>
+    <t>31</t>
   </si>
   <si>
     <t>W25Q32JVSSIQ</t>
@@ -589,7 +604,7 @@
     <t>C179173</t>
   </si>
   <si>
-    <t>31</t>
+    <t>32</t>
   </si>
   <si>
     <t>TPS564201DDCR</t>
@@ -604,7 +619,7 @@
     <t>C464812</t>
   </si>
   <si>
-    <t>32</t>
+    <t>33</t>
   </si>
   <si>
     <t>TYPE-C-31-M-12</t>
@@ -993,7 +1008,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="10" width="20" customWidth="1"/>
@@ -1653,19 +1668,19 @@
         <v>130</v>
       </c>
       <c r="E21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" t="s">
+        <v>129</v>
+      </c>
+      <c r="G21" t="s">
         <v>131</v>
       </c>
-      <c r="F21" t="s">
-        <v>41</v>
-      </c>
-      <c r="G21" t="s">
-        <v>129</v>
-      </c>
       <c r="H21" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" t="s">
         <v>132</v>
-      </c>
-      <c r="I21" t="s">
-        <v>133</v>
       </c>
       <c r="J21" t="s">
         <v>17</v>
@@ -1673,31 +1688,31 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B22">
+        <v>1</v>
+      </c>
+      <c r="C22" t="s">
         <v>134</v>
       </c>
-      <c r="B22">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>135</v>
       </c>
-      <c r="D22" t="s">
+      <c r="E22" t="s">
         <v>136</v>
-      </c>
-      <c r="E22" t="s">
-        <v>137</v>
       </c>
       <c r="F22" t="s">
         <v>41</v>
       </c>
       <c r="G22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="H22" t="s">
+        <v>137</v>
+      </c>
+      <c r="I22" t="s">
         <v>138</v>
-      </c>
-      <c r="I22" t="s">
-        <v>139</v>
       </c>
       <c r="J22" t="s">
         <v>17</v>
@@ -1705,31 +1720,31 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>139</v>
+      </c>
+      <c r="B23">
+        <v>1</v>
+      </c>
+      <c r="C23" t="s">
         <v>140</v>
       </c>
-      <c r="B23">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>141</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
         <v>142</v>
-      </c>
-      <c r="E23" t="s">
-        <v>143</v>
       </c>
       <c r="F23" t="s">
         <v>41</v>
       </c>
       <c r="G23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H23" t="s">
+        <v>143</v>
+      </c>
+      <c r="I23" t="s">
         <v>144</v>
-      </c>
-      <c r="I23" t="s">
-        <v>145</v>
       </c>
       <c r="J23" t="s">
         <v>17</v>
@@ -1737,28 +1752,28 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>145</v>
+      </c>
+      <c r="B24">
+        <v>1</v>
+      </c>
+      <c r="C24" t="s">
         <v>146</v>
       </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>147</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>148</v>
-      </c>
-      <c r="E24" t="s">
-        <v>149</v>
       </c>
       <c r="F24" t="s">
         <v>41</v>
       </c>
       <c r="G24" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H24" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="I24" t="s">
         <v>150</v>
@@ -1790,10 +1805,10 @@
         <v>152</v>
       </c>
       <c r="H25" t="s">
+        <v>149</v>
+      </c>
+      <c r="I25" t="s">
         <v>155</v>
-      </c>
-      <c r="I25" t="s">
-        <v>156</v>
       </c>
       <c r="J25" t="s">
         <v>17</v>
@@ -1801,31 +1816,31 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>156</v>
+      </c>
+      <c r="B26">
+        <v>1</v>
+      </c>
+      <c r="C26" t="s">
         <v>157</v>
       </c>
-      <c r="B26">
-        <v>1</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>158</v>
       </c>
-      <c r="D26" t="s">
+      <c r="E26" t="s">
         <v>159</v>
-      </c>
-      <c r="E26" t="s">
-        <v>160</v>
       </c>
       <c r="F26" t="s">
         <v>41</v>
       </c>
       <c r="G26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="H26" t="s">
+        <v>160</v>
+      </c>
+      <c r="I26" t="s">
         <v>161</v>
-      </c>
-      <c r="I26" t="s">
-        <v>162</v>
       </c>
       <c r="J26" t="s">
         <v>17</v>
@@ -1833,31 +1848,31 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>162</v>
+      </c>
+      <c r="B27">
+        <v>1</v>
+      </c>
+      <c r="C27" t="s">
         <v>163</v>
       </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>164</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>165</v>
-      </c>
-      <c r="E27" t="s">
-        <v>166</v>
       </c>
       <c r="F27" t="s">
         <v>41</v>
       </c>
       <c r="G27" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H27" t="s">
+        <v>166</v>
+      </c>
+      <c r="I27" t="s">
         <v>167</v>
-      </c>
-      <c r="I27" t="s">
-        <v>168</v>
       </c>
       <c r="J27" t="s">
         <v>17</v>
@@ -1865,28 +1880,28 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
+        <v>168</v>
+      </c>
+      <c r="B28">
+        <v>1</v>
+      </c>
+      <c r="C28" t="s">
         <v>169</v>
       </c>
-      <c r="B28">
-        <v>4</v>
-      </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>170</v>
       </c>
-      <c r="D28" t="s">
+      <c r="E28" t="s">
         <v>171</v>
-      </c>
-      <c r="E28" t="s">
-        <v>172</v>
       </c>
       <c r="F28" t="s">
         <v>41</v>
       </c>
       <c r="G28" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H28" t="s">
-        <v>54</v>
+        <v>172</v>
       </c>
       <c r="I28" t="s">
         <v>173</v>
@@ -1900,7 +1915,7 @@
         <v>174</v>
       </c>
       <c r="B29">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C29" t="s">
         <v>175</v>
@@ -1912,16 +1927,16 @@
         <v>177</v>
       </c>
       <c r="F29" t="s">
+        <v>41</v>
+      </c>
+      <c r="G29" t="s">
         <v>175</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
+        <v>54</v>
+      </c>
+      <c r="I29" t="s">
         <v>178</v>
-      </c>
-      <c r="H29" t="s">
-        <v>79</v>
-      </c>
-      <c r="I29" t="s">
-        <v>179</v>
       </c>
       <c r="J29" t="s">
         <v>17</v>
@@ -1929,31 +1944,31 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>179</v>
+      </c>
+      <c r="B30">
+        <v>1</v>
+      </c>
+      <c r="C30" t="s">
         <v>180</v>
       </c>
-      <c r="B30">
-        <v>1</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>181</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>182</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
+        <v>180</v>
+      </c>
+      <c r="G30" t="s">
         <v>183</v>
       </c>
-      <c r="F30" t="s">
-        <v>41</v>
-      </c>
-      <c r="G30" t="s">
-        <v>181</v>
-      </c>
       <c r="H30" t="s">
+        <v>79</v>
+      </c>
+      <c r="I30" t="s">
         <v>184</v>
-      </c>
-      <c r="I30" t="s">
-        <v>185</v>
       </c>
       <c r="J30" t="s">
         <v>17</v>
@@ -1961,31 +1976,31 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
+        <v>185</v>
+      </c>
+      <c r="B31">
+        <v>1</v>
+      </c>
+      <c r="C31" t="s">
         <v>186</v>
       </c>
-      <c r="B31">
-        <v>1</v>
-      </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>187</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>188</v>
-      </c>
-      <c r="E31" t="s">
-        <v>189</v>
       </c>
       <c r="F31" t="s">
         <v>41</v>
       </c>
       <c r="G31" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H31" t="s">
+        <v>189</v>
+      </c>
+      <c r="I31" t="s">
         <v>190</v>
-      </c>
-      <c r="I31" t="s">
-        <v>191</v>
       </c>
       <c r="J31" t="s">
         <v>17</v>
@@ -1993,28 +2008,28 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>191</v>
+      </c>
+      <c r="B32">
+        <v>1</v>
+      </c>
+      <c r="C32" t="s">
         <v>192</v>
       </c>
-      <c r="B32">
-        <v>1</v>
-      </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>193</v>
       </c>
-      <c r="D32" t="s">
+      <c r="E32" t="s">
         <v>194</v>
-      </c>
-      <c r="E32" t="s">
-        <v>195</v>
       </c>
       <c r="F32" t="s">
         <v>41</v>
       </c>
       <c r="G32" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H32" t="s">
-        <v>155</v>
+        <v>195</v>
       </c>
       <c r="I32" t="s">
         <v>196</v>
@@ -2046,7 +2061,7 @@
         <v>198</v>
       </c>
       <c r="H33" t="s">
-        <v>42</v>
+        <v>160</v>
       </c>
       <c r="I33" t="s">
         <v>201</v>
@@ -2055,8 +2070,40 @@
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>202</v>
+      </c>
+      <c r="B34">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>203</v>
+      </c>
+      <c r="D34" t="s">
+        <v>204</v>
+      </c>
+      <c r="E34" t="s">
+        <v>205</v>
+      </c>
+      <c r="F34" t="s">
+        <v>41</v>
+      </c>
+      <c r="G34" t="s">
+        <v>203</v>
+      </c>
+      <c r="H34" t="s">
+        <v>42</v>
+      </c>
+      <c r="I34" t="s">
+        <v>206</v>
+      </c>
+      <c r="J34" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>41</v>
       </c>
     </row>

</xml_diff>